<commit_message>
운동프로그램 갱신 2026-08-12 17:25:34.50
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v11.xlsx
+++ b/운동프로그램_6일_v11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0B58166-7E64-4AD7-95A9-E8FF2EFE7879}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDB15021-E3FD-460F-83CB-B76199137266}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
     <sheet name="복귀_일_등" sheetId="17" r:id="rId17"/>
     <sheet name="복귀_증량원칙" sheetId="18" r:id="rId18"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -16524,6 +16524,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -19172,7 +19176,7 @@
       </c>
       <c r="B23" s="72">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A23)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A23)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A23)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A23)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A23)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A23)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C23" s="68">
         <f>SUMIFS(간접계수맵!$F$7:$F$53,간접계수맵!$C$7:$C$53,$A23)</f>
@@ -19180,7 +19184,7 @@
       </c>
       <c r="D23" s="69">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E23" s="7" t="str">
         <f t="shared" si="1"/>
@@ -19222,12 +19226,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C25" s="74"/>
       <c r="D25" s="75">
         <f ca="1">SUM(D5:D24)</f>
-        <v>206.19</v>
+        <v>208.19</v>
       </c>
       <c r="E25" s="74" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21435,7 +21439,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>월_당기기A!$J$15+화_밀기A!$J$26+수_하체A!$J$23+목_당기기B!$J$14+금_밀기B!$J$29+토_하체B!$J$23</f>
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>57</v>
@@ -21811,7 +21815,7 @@
       </c>
       <c r="E7" s="27">
         <f>수_하체A!$E$23</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>104</v>
@@ -21874,7 +21878,7 @@
       </c>
       <c r="E10" s="27">
         <f>토_하체B!$E$23</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10" s="27" t="s">
         <v>125</v>
@@ -21909,7 +21913,7 @@
       <c r="D12" s="35"/>
       <c r="E12" s="34">
         <f>SUM(E5:E11)</f>
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -23265,7 +23269,7 @@
         <v>5</v>
       </c>
       <c r="E22" s="27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" s="33" t="s">
         <v>279</v>
@@ -23279,7 +23283,7 @@
       </c>
       <c r="J22" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K22,$E22,0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="42">
         <v>1</v>
@@ -23291,11 +23295,11 @@
       </c>
       <c r="E23" s="34">
         <f>SUM(E15:E22)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J23" s="41">
         <f>SUM(J15:J22)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -24647,7 +24651,7 @@
         <v>62</v>
       </c>
       <c r="E22" s="27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" s="33" t="s">
         <v>389</v>
@@ -24661,7 +24665,7 @@
       </c>
       <c r="J22" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K22,$E22,0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="42">
         <v>1</v>
@@ -24673,11 +24677,11 @@
       </c>
       <c r="E23" s="34">
         <f>SUM(E15:E22)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J23" s="41">
         <f>SUM(J15:J22)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1"/>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-12 19:22:10.67
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v11.xlsx
+++ b/운동프로그램_6일_v11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDB15021-E3FD-460F-83CB-B76199137266}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58E0F421-08ED-4E30-880A-00BF4A2BDE96}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -16524,10 +16524,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -19176,7 +19172,7 @@
       </c>
       <c r="B23" s="72">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A23)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A23)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A23)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A23)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A23)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A23)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C23" s="68">
         <f>SUMIFS(간접계수맵!$F$7:$F$53,간접계수맵!$C$7:$C$53,$A23)</f>
@@ -19184,7 +19180,7 @@
       </c>
       <c r="D23" s="69">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E23" s="7" t="str">
         <f t="shared" si="1"/>
@@ -19226,12 +19222,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C25" s="74"/>
       <c r="D25" s="75">
         <f ca="1">SUM(D5:D24)</f>
-        <v>208.19</v>
+        <v>207.19</v>
       </c>
       <c r="E25" s="74" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21439,7 +21435,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>월_당기기A!$J$15+화_밀기A!$J$26+수_하체A!$J$23+목_당기기B!$J$14+금_밀기B!$J$29+토_하체B!$J$23</f>
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>57</v>
@@ -21815,7 +21811,7 @@
       </c>
       <c r="E7" s="27">
         <f>수_하체A!$E$23</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>104</v>
@@ -21913,7 +21909,7 @@
       <c r="D12" s="35"/>
       <c r="E12" s="34">
         <f>SUM(E5:E11)</f>
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -23269,7 +23265,7 @@
         <v>5</v>
       </c>
       <c r="E22" s="27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" s="33" t="s">
         <v>279</v>
@@ -23283,7 +23279,7 @@
       </c>
       <c r="J22" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K22,$E22,0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K22" s="42">
         <v>1</v>
@@ -23295,11 +23291,11 @@
       </c>
       <c r="E23" s="34">
         <f>SUM(E15:E22)</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J23" s="41">
         <f>SUM(J15:J22)</f>
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-14 13:00:20.45
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v11.xlsx
+++ b/운동프로그램_6일_v11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58E0F421-08ED-4E30-880A-00BF4A2BDE96}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{9AF4581A-2CFF-4DDE-9A83-DA592B8C9F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6E5C7C0-C39F-4E01-BF45-D5277D0DBCBB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -16372,14 +16372,14 @@
     <xf numFmtId="0" fontId="46" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -16522,6 +16522,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17266,28 +17270,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="96" t="s">
         <v>393</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="96" t="s">
+      <c r="A4" s="97" t="s">
         <v>394</v>
       </c>
-      <c r="B4" s="96"/>
-      <c r="C4" s="96"/>
-      <c r="D4" s="96"/>
-      <c r="E4" s="96"/>
-      <c r="F4" s="96"/>
-      <c r="G4" s="96"/>
-      <c r="H4" s="96"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="A6" s="56" t="s">
@@ -17554,11 +17558,11 @@
       </c>
       <c r="E15" s="59">
         <f t="shared" ca="1" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" s="60">
         <f t="shared" ca="1" si="1"/>
-        <v>1.32</v>
+        <v>0.99</v>
       </c>
       <c r="G15" s="61" t="s">
         <v>404</v>
@@ -18637,7 +18641,7 @@
       </c>
       <c r="F54" s="66">
         <f ca="1">SUM(F7:F53)</f>
-        <v>55.190000000000005</v>
+        <v>54.860000000000007</v>
       </c>
     </row>
   </sheetData>
@@ -18716,7 +18720,7 @@
       <c r="F5" s="67" t="s">
         <v>461</v>
       </c>
-      <c r="G5" s="97" t="s">
+      <c r="G5" s="95" t="s">
         <v>462</v>
       </c>
       <c r="H5" s="70">
@@ -18747,7 +18751,7 @@
       <c r="F6" s="67" t="s">
         <v>463</v>
       </c>
-      <c r="G6" s="97"/>
+      <c r="G6" s="95"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
       <c r="A7" s="67" t="s">
@@ -18772,7 +18776,7 @@
       <c r="F7" s="67" t="s">
         <v>464</v>
       </c>
-      <c r="G7" s="97" t="s">
+      <c r="G7" s="95" t="s">
         <v>465</v>
       </c>
       <c r="H7" s="70">
@@ -18803,7 +18807,7 @@
       <c r="F8" s="67" t="s">
         <v>466</v>
       </c>
-      <c r="G8" s="97"/>
+      <c r="G8" s="95"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
       <c r="A9" s="67" t="s">
@@ -18828,7 +18832,7 @@
       <c r="F9" s="67" t="s">
         <v>467</v>
       </c>
-      <c r="G9" s="97"/>
+      <c r="G9" s="95"/>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
       <c r="A10" s="67" t="s">
@@ -18853,7 +18857,7 @@
       <c r="F10" s="67" t="s">
         <v>468</v>
       </c>
-      <c r="G10" s="97"/>
+      <c r="G10" s="95"/>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
       <c r="A11" s="67" t="s">
@@ -19033,7 +19037,7 @@
       <c r="F17" s="67" t="s">
         <v>474</v>
       </c>
-      <c r="G17" s="97" t="s">
+      <c r="G17" s="95" t="s">
         <v>254</v>
       </c>
       <c r="H17" s="70">
@@ -19064,7 +19068,7 @@
       <c r="F18" s="67" t="s">
         <v>475</v>
       </c>
-      <c r="G18" s="97"/>
+      <c r="G18" s="95"/>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1">
       <c r="A19" s="67" t="s">
@@ -19097,7 +19101,7 @@
       </c>
       <c r="B20" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A20)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A20)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A20)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A20)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A20)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A20)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" s="68">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$53,간접계수맵!$C$7:$C$53,$A20)</f>
@@ -19105,7 +19109,7 @@
       </c>
       <c r="D20" s="69">
         <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -19147,19 +19151,19 @@
       </c>
       <c r="B22" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A22)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A22)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A22)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A22)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A22)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A22)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C22" s="68">
         <f ca="1">SUMIFS(간접계수맵!$F$7:$F$53,간접계수맵!$C$7:$C$53,$A22)</f>
-        <v>2.31</v>
+        <v>1.98</v>
       </c>
       <c r="D22" s="69">
         <f t="shared" ca="1" si="0"/>
-        <v>10.31</v>
+        <v>8.98</v>
       </c>
       <c r="E22" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>충분</v>
+        <v>하한</v>
       </c>
       <c r="F22" s="67" t="s">
         <v>479</v>
@@ -19222,12 +19226,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C25" s="74"/>
       <c r="D25" s="75">
         <f ca="1">SUM(D5:D24)</f>
-        <v>207.19</v>
+        <v>204.85999999999999</v>
       </c>
       <c r="E25" s="74" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21435,7 +21439,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>월_당기기A!$J$15+화_밀기A!$J$26+수_하체A!$J$23+목_당기기B!$J$14+금_밀기B!$J$29+토_하체B!$J$23</f>
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>57</v>
@@ -21769,7 +21773,7 @@
       </c>
       <c r="E5" s="27">
         <f>월_당기기A!$E$15</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>104</v>
@@ -21909,7 +21913,7 @@
       <c r="D12" s="35"/>
       <c r="E12" s="34">
         <f>SUM(E5:E11)</f>
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -22309,7 +22313,7 @@
         <v>5</v>
       </c>
       <c r="E11" s="27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" s="33" t="s">
         <v>173</v>
@@ -22325,7 +22329,7 @@
       </c>
       <c r="J11" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K11,$E11,0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" s="42">
         <v>1</v>
@@ -22345,7 +22349,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" s="33" t="s">
         <v>199</v>
@@ -22359,7 +22363,7 @@
       </c>
       <c r="J12" s="41">
         <f>IF(볼륨램프!$C$4&gt;=$K12,$E12,0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" s="42">
         <v>1</v>
@@ -22441,11 +22445,11 @@
       </c>
       <c r="E15" s="45">
         <f>SUM(E6:E14)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J15" s="46">
         <f>SUM(J6:J14)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>